<commit_message>
Updated Kevin worklog 3/4/2026
</commit_message>
<xml_diff>
--- a/Work_Log/Kevin_Hours_Log.xlsx
+++ b/Work_Log/Kevin_Hours_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\K_Documents\CEN4908C\Senior_Design_TI_Project\Work_Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AE86FC-3396-467B-955C-5F6944B25669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52CB9B9-82EC-4333-A4F1-74F11DD982F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="8170" xr2:uid="{1E1DE2E1-E43F-4C7B-805F-E7F882405594}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
   <si>
     <t>Kevin Su Senior Design Work Log</t>
   </si>
@@ -129,6 +129,15 @@
   </si>
   <si>
     <t>Assistem with data collection and ML model improvement suggestions.</t>
+  </si>
+  <si>
+    <t>Began redesigning PCB schematic for a Raspberry PI 4 backpack/peripheral.</t>
+  </si>
+  <si>
+    <t>Completed PCB schematic redesign for a Raspberry PI 4 backpack/peripheral.</t>
+  </si>
+  <si>
+    <t>Fixed wiring issues identified by Altium tool.</t>
   </si>
 </sst>
 </file>
@@ -542,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5815A0D-EF96-486C-AACC-708D8CEA56AE}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.6328125" customWidth="1"/>
@@ -1067,13 +1076,73 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="E27" s="4">
-        <v>0.79166666666666663</v>
+        <v>0.8125</v>
       </c>
       <c r="F27" s="5">
-        <v>8.3333333333333329E-2</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="3">
+        <v>46084</v>
+      </c>
+      <c r="D28" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E28" s="4">
+        <v>0.875</v>
+      </c>
+      <c r="F28" s="5">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="3">
+        <v>46085</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0.65625</v>
+      </c>
+      <c r="E29" s="4">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F29" s="5">
+        <v>5.2083333333333336E-2</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="3">
+        <v>46085</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E30" s="4">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F30" s="5">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Kevin Work hours
</commit_message>
<xml_diff>
--- a/Work_Log/Kevin_Hours_Log.xlsx
+++ b/Work_Log/Kevin_Hours_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\K_Documents\CEN4908C\Senior_Design_TI_Project\Work_Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52CB9B9-82EC-4333-A4F1-74F11DD982F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40FB9D77-DA80-4934-ADEE-A372EF7C3C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="8170" xr2:uid="{1E1DE2E1-E43F-4C7B-805F-E7F882405594}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="8170" xr2:uid="{1E1DE2E1-E43F-4C7B-805F-E7F882405594}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="37">
   <si>
     <t>Kevin Su Senior Design Work Log</t>
   </si>
@@ -138,6 +138,15 @@
   </si>
   <si>
     <t>Fixed wiring issues identified by Altium tool.</t>
+  </si>
+  <si>
+    <t>Began placement of PCB components.</t>
+  </si>
+  <si>
+    <t>Worked on placing PCB components.</t>
+  </si>
+  <si>
+    <t>Completed PCB component placement and began routing.</t>
   </si>
 </sst>
 </file>
@@ -551,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5815A0D-EF96-486C-AACC-708D8CEA56AE}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.6328125" customWidth="1"/>
@@ -1145,6 +1154,66 @@
         <v>33</v>
       </c>
     </row>
+    <row r="31" spans="2:7" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="3">
+        <v>46097</v>
+      </c>
+      <c r="D31" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="E31" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="F31" s="5">
+        <v>0.125</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B32" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="3">
+        <v>46098</v>
+      </c>
+      <c r="D32" s="4">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0.875</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B33" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="3">
+        <v>46099</v>
+      </c>
+      <c r="D33" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="E33" s="4">
+        <v>0.875</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0.25</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Kevin Work log
</commit_message>
<xml_diff>
--- a/Work_Log/Kevin_Hours_Log.xlsx
+++ b/Work_Log/Kevin_Hours_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\K_Documents\CEN4908C\Senior_Design_TI_Project\Work_Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D39A5B-D954-48EF-9CCB-5707CBF51F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660654F4-E0CD-464C-B752-ACC182AAE622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1E1DE2E1-E43F-4C7B-805F-E7F882405594}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="46">
   <si>
     <t>Kevin Su Senior Design Work Log</t>
   </si>
@@ -187,6 +187,15 @@
   </si>
   <si>
     <t xml:space="preserve">Continuted working PCB design for a 4 layer design. Continued routing netlist signals. Created GND plane. </t>
+  </si>
+  <si>
+    <t>Completed 4 Layer PCB for review.</t>
+  </si>
+  <si>
+    <t>6:45:00PM</t>
+  </si>
+  <si>
+    <t>Completed code for SPI to transmit data from mmWaveradar.</t>
   </si>
 </sst>
 </file>
@@ -658,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5815A0D-EF96-486C-AACC-708D8CEA56AE}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.6328125" customWidth="1"/>
@@ -1432,10 +1441,48 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:9" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B40" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="3">
+        <v>46107</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E40" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="F40" s="5">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="I40" t="e" vm="1">
         <f>_xleta.SUM</f>
         <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="3">
+        <v>46119</v>
+      </c>
+      <c r="D41" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0.19791666666666666</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>